<commit_message>
Consolidate SK13102 summary under single HS code 8531202000
All items are fishing bite alarms/receivers from one sender; per the
SK13102-CZ instruction doc the whole shipment is declared under
8531202000 (Rybarske alarmy) instead of splitting by the invoice's
8531202090.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SkpngkaLv73LdC3QLgM1Vp
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Sonik_Sports_SK13102.xlsx
+++ b/output/HS_Code_Summary_Sonik_Sports_SK13102.xlsx
@@ -472,19 +472,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -548,11 +547,6 @@
           <t>Antidumping</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -567,20 +561,20 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Rybářské alarmy (Fishing alarms – alarm sets + bivvy lamp)</t>
+          <t>Rybářské alarmy (Fishing bite alarms – sety s bivvy lampou, single alarmy a přijímače, SKS2 / GIZMO2)</t>
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>1315.6</v>
+        <v>1603.6</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>1477</v>
+        <v>1803.6</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>1930</v>
+        <v>2670</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>168466.1</v>
+        <v>200293.2</v>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
@@ -592,91 +586,48 @@
           <t>Ne / N.A.</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>HS + česká descripce dle dokladu SK13102-CZ (HC0083, HC0087, HC0088, HC0089)</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Fishing Capital Company Limited, Weihai, China</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>8531202090</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Fishing Bite Alarm / Receiver (single alarmy a přijímače – česká descripce v dokladech není)</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>288</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>326.6</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>740</v>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>31827.1</v>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>Ne / N.A.</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>Ne / N.A.</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>HS dle faktury TD25110 (HC0080, HC0081, HC0082, HC0084, HC0085, HC0086)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr"/>
-      <c r="C7" s="8" t="inlineStr"/>
-      <c r="D7" s="10" t="n">
+      <c r="B6" s="9" t="inlineStr"/>
+      <c r="C6" s="8" t="inlineStr"/>
+      <c r="D6" s="10" t="n">
         <v>1603.6</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E6" s="10" t="n">
         <v>1803.6</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F6" s="9" t="n">
         <v>2670</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G6" s="10" t="n">
         <v>200293.2</v>
       </c>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
-      <c r="J7" s="8" t="inlineStr"/>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr"/>
+      <c r="I6" s="9" t="inlineStr"/>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>POZNÁMKY / NOTES</t>
         </is>
       </c>
     </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>⚠ PREFERENČNÍ VĚTA: NENÍ v dokladech. Původ zboží: P.R.C. (Čína) – preferenční původ se neuplatní, platí standardní celní sazba třetí země.</t>
+        </is>
+      </c>
+    </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>⚠ PREFERENČNÍ VĚTA: NENÍ v dokladech. Původ zboží: P.R.C. (Čína) – preferenční původ se neuplatní, platí standardní celní sazba třetí země.</t>
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>HS kód: faktura TD25110 uvádí u všech položek 8531202090; dle dokladu SK13102-CZ deklarováno vše pod 8531202000 (rybářské alarmy) – jeden HS kód pro celou zásilku, jeden odesílatel.</t>
         </is>
       </c>
     </row>
@@ -690,48 +641,41 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>HC0081 (SKS2 RECEIVER, 40 ks) a HC0086 (GIZMO2 RECEIVER, 30 ks) nemají v packing listu samostatné váhy – baleno v kartonech s HC0080 / HC0085; jejich váha je zahrnuta v řádku 8531202090.</t>
+          <t>HC0081 (SKS2 RECEIVER, 40 ks) a HC0086 (GIZMO2 RECEIVER, 30 ks) nemají v packing listu samostatné váhy – baleno v kartonech s HC0080 / HC0085; váha zahrnuta v celkovém součtu.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>Rozpor HS: faktura uvádí 8531202090 pro všechny položky; doklad SK13102-CZ uvádí 8531202000 pro sety HC0083/HC0087/HC0088/HC0089 – použit doklad SK13102-CZ (má přednost).</t>
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>B/L uvádí i FISHING RODS a 348 CTNS / 3 954,8 kg / 57,518 CBM – CI/PL TD25110 pokrývá 241 CTNS / 1 803,6 kg. Pruty a zbytek kontejneru nejsou v této faktuře (T1 bude doplněna dle e-mailu).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>B/L uvádí i FISHING RODS a 348 CTNS / 3 954,8 kg / 57,518 CBM – CI/PL TD25110 pokrývá 241 CTNS / 1 803,6 kg. Pruty a zbytek kontejneru nejsou v této faktuře (T1 bude doplněna dle e-mailu).</t>
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Sleva: žádná obchodní sleva na faktuře – proporcionální rozpočet slevy se neuplatní. CBAM: nevztahuje se. Antidumping: na HS 8531 20 z Číny se nevztahuje.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Sleva: žádná obchodní sleva na faktuře – proporcionální rozpočet slevy se neuplatní. CBAM: nevztahuje se. Antidumping: na HS 8531 20 z Číny se nevztahuje.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
           <t>Trasa: Qingdao → Koper (COSCO SHIPPING SOLAR 036W), kontejner OOCU6435613, na palubě 08.05.2026. Předpokládaný příjezd Kněževes: 20.07.2026.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A14:J14"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="A15:J15"/>
-    <mergeCell ref="A16:J16"/>
-    <mergeCell ref="A10:J10"/>
-    <mergeCell ref="A13:J13"/>
-    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A8:I8"/>
+    <mergeCell ref="A12:I12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Use TARIC code 8531202090 for SK13102 summary
Confirmed in TARIC: CN 8531 20 20 splits into 8531202010 (civil
aircraft) and 8531202090 (other), so 8531202090 from the invoice is the
correct declarable 10-digit code; 8531202000 from the instruction doc
was the 8-digit code padded with zeros.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SkpngkaLv73LdC3QLgM1Vp
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Sonik_Sports_SK13102.xlsx
+++ b/output/HS_Code_Summary_Sonik_Sports_SK13102.xlsx
@@ -500,7 +500,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -556,7 +555,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>8531202000</t>
+          <t>8531202090</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -610,6 +609,7 @@
       <c r="H6" s="9" t="inlineStr"/>
       <c r="I6" s="9" t="inlineStr"/>
     </row>
+    <row r="7"/>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
         <is>
@@ -627,7 +627,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>HS kód: faktura TD25110 uvádí u všech položek 8531202090; dle dokladu SK13102-CZ deklarováno vše pod 8531202000 (rybářské alarmy) – jeden HS kód pro celou zásilku, jeden odesílatel.</t>
+          <t>HS kód: celá zásilka deklarována pod TARIC 8531202090 (CN 8531 20 20 – návěstní panely s LED, Ostatní) dle faktury TD25110, potvrzeno v TARIC. Doklad SK13102-CZ uvádí 8531202000 – to je 8místný kód doplněný nulami, na 10místné úrovni platí 8531202090.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild SK13102 summary from the three final invoice sets
TD2026086 (fishing rods), TD2026099 (feeders) and TD2026104 (alarm
sets) replace the earlier TD25110/SK11931-UK data, which does not
belong to this container. Three HS rows under one sender: 9507100000,
9507900000 (both proposed, not in docs - flagged) and 8531202090.
Totals reconcile with B/L QDSE2602385: 348 CTNS, 57.518 CBM,
3,954.75 kg GW, USD 179,239.70.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SkpngkaLv73LdC3QLgM1Vp
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Sonik_Sports_SK13102.xlsx
+++ b/output/HS_Code_Summary_Sonik_Sports_SK13102.xlsx
@@ -472,18 +472,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,10 +498,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Invoice TD25110 (POR001978-UK + POR002049-UK) · B/L QDSE2602385 · Container OOCU6435613 · Qingdao → Koper</t>
-        </is>
-      </c>
-    </row>
+          <t>Invoices TD2026086 + TD2026099 + TD2026104 · B/L QDSE2602385 · Container OOCU6435613 (40'HC) · Qingdao → Koper · souhrn sedí na B/L: 348 CTNS / 57,518 CBM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -508,42 +511,52 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
           <t>HS code</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Net weight (kg)</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Gross weight (kg)</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Quantity (pcs)</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Customs value (USD)</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>CBAM</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Antidumping</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
@@ -555,127 +568,236 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
+          <t>TD2026086</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>9507100000</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Rybářské pruty (Fishing rods – HEROX, KRAFT, XTRACTOR CUSTOM, TURBOSPOD; POR002138, POR002332, POR002411)</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>1721.35</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>3403.15</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>5440</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>108853</v>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Ne / N.A.</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Ne / N.A.</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>HS není v dokladech – zařazeno námi: CN 9507 10 00 rybářské pruty. OVĚŘIT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Fishing Capital Company Limited, Weihai, China</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>TD2026099</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>9507900000</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Krmítka (NYTRO ARYZON Continental Feeder 1oz/2oz; POR002411)</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Ne / N.A.</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>Ne / N.A.</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>HS není v dokladech – zařazeno námi: CN 9507 90 00 ostatní rybářské potřeby. OVĚŘIT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Fishing Capital Company Limited, Weihai, China</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>TD2026104</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
           <t>8531202090</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Rybářské alarmy (Fishing bite alarms – sety s bivvy lampou, single alarmy a přijímače, SKS2 / GIZMO2)</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>1603.6</v>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>1803.6</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>2670</v>
-      </c>
-      <c r="G5" s="7" t="n">
-        <v>200293.2</v>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Rybářské alarmy (Fishing bite alarm sety + bivvy lampa, SKS2 / GIZMO2; POR002365, POR002411)</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>504.5</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>551</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>750</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>70285.5</v>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>Ne / N.A.</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>Ne / N.A.</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>HS dle dokladu SK13102-CZ (8531 20 20), TARIC 8531202090 potvrzen; česká descripce z dokladu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr"/>
-      <c r="C6" s="8" t="inlineStr"/>
-      <c r="D6" s="10" t="n">
-        <v>1603.6</v>
-      </c>
-      <c r="E6" s="10" t="n">
-        <v>1803.6</v>
-      </c>
-      <c r="F6" s="9" t="n">
-        <v>2670</v>
-      </c>
-      <c r="G6" s="10" t="n">
-        <v>200293.2</v>
-      </c>
-      <c r="H6" s="9" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
-    </row>
-    <row r="7"/>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr"/>
+      <c r="C8" s="9" t="inlineStr"/>
+      <c r="D8" s="8" t="inlineStr"/>
+      <c r="E8" s="10" t="n">
+        <v>2226.25</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>3954.75</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>6230</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>179239.7</v>
+      </c>
+      <c r="I8" s="9" t="inlineStr"/>
+      <c r="J8" s="9" t="inlineStr"/>
+      <c r="K8" s="8" t="inlineStr"/>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>POZNÁMKY / NOTES</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>⚠ PREFERENČNÍ VĚTA: NENÍ v dokladech. Původ zboží: P.R.C. (Čína) – preferenční původ se neuplatní, platí standardní celní sazba třetí země.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>HS kód: celá zásilka deklarována pod TARIC 8531202090 (CN 8531 20 20 – návěstní panely s LED, Ostatní) dle faktury TD25110, potvrzeno v TARIC. Doklad SK13102-CZ uvádí 8531202000 – to je 8místný kód doplněný nulami, na 10místné úrovni platí 8531202090.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>Dopravné (dle e-mailu): 4 250 USD, FOB QINGDAO – přičíst k celní hodnotě při deklaraci (není zahrnuto ve fakturní hodnotě výše).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>HC0081 (SKS2 RECEIVER, 40 ks) a HC0086 (GIZMO2 RECEIVER, 30 ks) nemají v packing listu samostatné váhy – baleno v kartonech s HC0080 / HC0085; váha zahrnuta v celkovém součtu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>B/L uvádí i FISHING RODS a 348 CTNS / 3 954,8 kg / 57,518 CBM – CI/PL TD25110 pokrývá 241 CTNS / 1 803,6 kg. Pruty a zbytek kontejneru nejsou v této faktuře (T1 bude doplněna dle e-mailu).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>⚠ PREFERENČNÍ VĚTA: NENÍ v žádném z dokladů. Původ zboží: P.R.C. (Čína) – preferenční původ se neuplatní, platí standardní celní sazba třetí země.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>⚠ HS kódy 9507100000 (pruty) a 9507900000 (krmítka) NEJSOU v obchodních dokladech – navrženy dle sazebníku, před podáním JSD ověřit. Pouze alarmy (8531202090) mají HS doložen dokladem SK13102-CZ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Kontrola vs. B/L: 272+1+75 = 348 CTNS ✓; 54,052+0,010+3,456 = 57,518 CBM ✓; GW 3 403,15+0,60+551,00 = 3 954,75 kg vs. B/L 3 954,80 kg (rozdíl 0,05 kg – zaokrouhlení).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>Sleva: žádná obchodní sleva na faktuře – proporcionální rozpočet slevy se neuplatní. CBAM: nevztahuje se. Antidumping: na HS 8531 20 z Číny se nevztahuje.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+          <t>Faktura TD25110 / SK11931-UK z dřívějšího podkladu do tohoto kontejneru NEPATŘÍ – nahrazena třemi sadami dokladů výše (e-mail V. Majer 20.07.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Trasa: Qingdao → Koper (COSCO SHIPPING SOLAR 036W), kontejner OOCU6435613, na palubě 08.05.2026. Předpokládaný příjezd Kněževes: 20.07.2026.</t>
+          <t>Dopravné (dle e-mailu): 4 250 USD, FOB QINGDAO – přičíst k celní hodnotě při deklaraci (není zahrnuto ve fakturních hodnotách výše).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Sleva: žádná obchodní sleva – proporcionální rozpočet se neuplatní. CBAM: nevztahuje se. Antidumping: na HS 9507 ani 8531 20 z Číny se aktuálně nevztahuje. Bez dřevěného obalového materiálu (prohlášení na fakturách).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Trasa: Qingdao → Koper (COSCO SHIPPING SOLAR 036W), kontejner OOCU6435613 / seal NK037870, na palubě 08.05.2026. Dále tahačem, předpokládaný příjezd Kněževes: 20.07.2026. T1 bude doplněna.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A11:I11"/>
-    <mergeCell ref="A10:I10"/>
-    <mergeCell ref="A13:I13"/>
-    <mergeCell ref="A14:I14"/>
-    <mergeCell ref="A9:I9"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A12:K12"/>
+    <mergeCell ref="A15:K15"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A11:K11"/>
+    <mergeCell ref="A10:K10"/>
+    <mergeCell ref="A13:K13"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A17:K17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>